<commit_message>
Update holdings and staking Excel reports
Refresh two Excel reports: Changes_in_the_Number_of_Holdings.xlsx and Numerai_data_staking_sumarry.xlsx. These are binary workbook updates (data refresh/edits), so contents are not shown in the diff; likely updated holdings counts and Numerai staking summary data.
</commit_message>
<xml_diff>
--- a/Changes_in_the_Number_of_Holdings.xlsx
+++ b/Changes_in_the_Number_of_Holdings.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moda2\OneDrive\デスクトップ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moda2\Projects\Holdings-of-Numerai-GP-LLC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{195FE4DC-E4AA-4EF6-8FBC-FAC2D89CF20A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288C6380-08B8-4AD5-A934-B53C15EC11BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-72" yWindow="-13068" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Change History" sheetId="2" r:id="rId1"/>
     <sheet name="Long Positions and Holdings" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'Long Positions and Holdings'!$A$1:$C$13</definedName>
+    <definedName name="ExternalData_1" localSheetId="1" hidden="1">'Long Positions and Holdings'!$A$1:$C$14</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,26 +46,26 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>Modifier</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="4"/>
   </si>
   <si>
     <t>Modification Date and Time</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="4"/>
   </si>
   <si>
     <t>Comments</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="4"/>
   </si>
   <si>
     <t>Kei Sanada</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="4"/>
   </si>
   <si>
     <t>Create a new file</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="4"/>
   </si>
   <si>
     <t>Date</t>
@@ -75,7 +75,11 @@
   </si>
   <si>
     <t>Long positions(1B)</t>
-    <phoneticPr fontId="2"/>
+    <phoneticPr fontId="3"/>
+  </si>
+  <si>
+    <t>Update</t>
+    <phoneticPr fontId="3"/>
   </si>
 </sst>
 </file>
@@ -85,12 +89,20 @@
   <numFmts count="1">
     <numFmt numFmtId="26" formatCode="\$#,##0.00_);[Red]\(\$#,##0.00\)"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Yu Gothic"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+      <charset val="128"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -135,23 +147,26 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="26" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -243,7 +258,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="ja-JP"/>
+          <a:endParaRPr lang="ja-JP" altLang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -280,10 +295,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'Long Positions and Holdings'!$A$2:$A$13</c:f>
+              <c:f>'Long Positions and Holdings'!$A$2:$A$14</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>44926</c:v>
                 </c:pt>
@@ -319,16 +334,19 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>45930</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46022</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Long Positions and Holdings'!$B$2:$B$13</c:f>
+              <c:f>'Long Positions and Holdings'!$B$2:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>\$#,##0.00_);[Red]\(\$#,##0.00\)</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>0.15</c:v>
                 </c:pt>
@@ -364,6 +382,9 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0.71</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.83</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -429,10 +450,10 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'Long Positions and Holdings'!$A$2:$A$13</c:f>
+              <c:f>'Long Positions and Holdings'!$A$2:$A$14</c:f>
               <c:numCache>
                 <c:formatCode>m/d/yyyy</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>44926</c:v>
                 </c:pt>
@@ -468,16 +489,19 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>45930</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46022</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Long Positions and Holdings'!$C$2:$C$13</c:f>
+              <c:f>'Long Positions and Holdings'!$C$2:$C$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>111</c:v>
                 </c:pt>
@@ -513,6 +537,9 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>546</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>608</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -582,6 +609,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="697731536"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="0"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -640,6 +668,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="697733936"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
@@ -696,6 +725,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="526668336"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblOffset val="100"/>
         <c:baseTimeUnit val="months"/>
@@ -1393,7 +1423,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{671D2D16-4D92-49CE-95B3-65847F4E2ECA}" name="holdings_LongPosition" displayName="holdings_LongPosition" ref="A1:C13" tableType="queryTable" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{671D2D16-4D92-49CE-95B3-65847F4E2ECA}" name="holdings_LongPosition" displayName="holdings_LongPosition" ref="A1:C14" tableType="queryTable" totalsRowShown="0">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5A15CF49-09C3-4843-82D9-4B300E3C334D}" uniqueName="1" name="Date" queryTableFieldId="1" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{67AA2156-28B6-4F3B-820E-BC80D61A32BA}" uniqueName="2" name="Long positions(1B)" queryTableFieldId="2" dataDxfId="0"/>
@@ -1698,7 +1728,15 @@
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="B3" s="2"/>
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2">
+        <v>46076</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="4" spans="1:3">
       <c r="B4" s="2"/>
@@ -1725,14 +1763,14 @@
       <c r="C9" s="3"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="2"/>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E09DF5A6-16E4-4C64-AFB2-5D67963E4C25}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="11.25" bestFit="1" customWidth="1"/>
@@ -1883,8 +1921,19 @@
         <v>546</v>
       </c>
     </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="4">
+        <v>46022</v>
+      </c>
+      <c r="B14" s="5">
+        <v>0.83</v>
+      </c>
+      <c r="C14">
+        <v>608</v>
+      </c>
+    </row>
   </sheetData>
-  <phoneticPr fontId="2"/>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>